<commit_message>
data update again, added CYBR 5830 as topic choice
</commit_message>
<xml_diff>
--- a/cirt_data.xlsx
+++ b/cirt_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ce1ebde9cded71ae/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="166" documentId="13_ncr:1_{C6350078-5CFC-4B20-8D31-D68148B331D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A0E237A-3892-4FBD-ABF0-177C512E6849}"/>
+  <xr:revisionPtr revIDLastSave="381" documentId="13_ncr:1_{C6350078-5CFC-4B20-8D31-D68148B331D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7652BA7E-9D2A-4F39-991C-96B793DF97D0}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{969D6A76-162A-4286-A653-6BBA36AECB0D}"/>
+    <workbookView xWindow="-16365" yWindow="-165" windowWidth="16530" windowHeight="28410" xr2:uid="{969D6A76-162A-4286-A653-6BBA36AECB0D}"/>
   </bookViews>
   <sheets>
     <sheet name="courses" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8333" uniqueCount="2616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8381" uniqueCount="2640">
   <si>
     <t>Effective Communication: Writing</t>
   </si>
@@ -7886,6 +7886,78 @@
   </si>
   <si>
     <t>Fall 2026, Spring 2026, Spring 2025, Fall 2024-DTSC only</t>
+  </si>
+  <si>
+    <t>None during Fall 2024-Fall 2026</t>
+  </si>
+  <si>
+    <t>Fall 2026, Summer 2026, Spring 2026, Fall 2025, Summer 2025, Spring 2025, Fall 2024</t>
+  </si>
+  <si>
+    <t>Fall 2026, Spring 2026</t>
+  </si>
+  <si>
+    <t>Spring 2026, Fall 2025</t>
+  </si>
+  <si>
+    <t>Summer 2026, Fall 2025, Spring 2025</t>
+  </si>
+  <si>
+    <t>Fall 2026, Spring 2026, Summer 2025, Spring 2025, Fall 2024</t>
+  </si>
+  <si>
+    <t>Fall 2026, Spring 2026, Fall 2025, Summer 2025</t>
+  </si>
+  <si>
+    <t>Summer 2026, Fall 2025, Summer 2025, Spring 2025, Fall 2024</t>
+  </si>
+  <si>
+    <t>Fall 2026, Spring 2026, Summer 2025, Fall 2024</t>
+  </si>
+  <si>
+    <t>Fall 2026, Fall 2025, Spring 2025, Fall 2024</t>
+  </si>
+  <si>
+    <t>Spring 2026, Spring 2025, Fall 2024</t>
+  </si>
+  <si>
+    <t>Summer 2026, Summer 2025</t>
+  </si>
+  <si>
+    <t>Spring 2026, Fall 2025, Spring 2025</t>
+  </si>
+  <si>
+    <t>CYBR-5830-2257-001</t>
+  </si>
+  <si>
+    <t>Fall 2025, Spring 2025, Fall 2024</t>
+  </si>
+  <si>
+    <t>CYBR-5830-2251-002</t>
+  </si>
+  <si>
+    <t>CYBR-5830-2247-003</t>
+  </si>
+  <si>
+    <t>Embedded Cybersecurity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Embedded devices and IoT are all around us - they are involved in our nation's most critical infrastructure and industries, as well as deployed commonly across households and in businesses of all sizes. Such devices are known as Operational Technology (OT) – OT is vastly different from Information Technology (IT). Similarly, securing such products through OT security is worlds apart from IT security, the normal intention behind the term “cybersecurity”. The goal of this course is to expose students to a wide array of technologies, techniques, concepts, and regulations that are applicable to the world around them and valuable in their future security careers, regardless of where they end up. In this course, students should expect to learn the basics of secure product development and embedded/IoT systems, as well as cover the following additional topics: Asset threat modeling and design vulnerability assessment; Security testing and verification to identify implementation vulnerabilities (penetration testing, static analysis, fuzz testing, input/unit boundary analysis, etc.); Hardware hacking, reverse engineering, serial and wireless communications sniffing, side channel attacks (fault injection and power monitoring), and more; Post-market sales, implementation, maintenance, and End-of-Life/End-of-Service (Software Bill of Materials, VeX, Instructions for Use, in-field software updates, disclosures, agreements, etc.); Product security governance (organizational policies and procedures); and Global and U.S.-based product security regulatory and consensus standards (ISO/IEC, FDA, HSCC, Executive Orders, GDPR, HIPAA, MDR, AAMI, etc.) </t>
+  </si>
+  <si>
+    <t>The class will be a mixture of lecture, hands-on exercises, guest lectures from industry experts, and group learning and projects. NO PREREQUISITES ARE REQUIRED FOR THIS COURSE. All content and knowledge base required to be successful in this course will be covered and provided by the instructor. Optional textbooks can supplement the course, but no textbooks are required. All equipment needed will similarly be provided, except students will be expected to bring their own laptop.</t>
+  </si>
+  <si>
+    <t>Embedded devices and IoT are all around us - they are involved in our nation's most critical infrastructure and industries, as well as deployed commonly across households and in businesses of all sizes. Such devices are known as Operational Technology (OT) – OT is vastly different from Information Technology (IT). Similarly, securing such products through OT security is worlds apart from IT security, the normal intention behind the term “cybersecurity”. The goal of this course is to expose students to a wide array of technologies, techniques, concepts, and regulations that are applicable to the world around them and valuable in their future security or engineering careers, regardless of where they end up. In this course, students should expect to learn the basics of secure product development and embedded/IoT systems, as well as cover the following additional topics: Asset threat modeling and design vulnerability assessment; Security testing and verification to identify implementation vulnerabilities (penetration testing, static analysis, fuzz testing, software composition analysis, attack surface analysis, etc.); Hardware hacking, reverse engineering, serial and wireless communications sniffing, side channel attacks (fault injection and power monitoring), and more; Post-market sales, implementation, maintenance, and End-of-Life/End-of-Service (Software Bill of Materials, VEX, Instructions for Use, in-field software updates, disclosures, agreements, etc.); Product security governance (organizational policies and procedures); and Global and U.S.-based product security regulatory and consensus standards (ISO/IEC, FDA, HSCC, Executive Orders, GDPR, HIPAA, MDR, AAMI, etc.)</t>
+  </si>
+  <si>
+    <t>The class will be a mixture of lecture, hands-on exercises, guest lectures from industry experts, and group learning and projects. NO PREREQUISITES ARE REQUIRED FOR THIS COURSE. All content and knowledge base required to be successful in this course will be covered and provided by the instructor. Optional textbooks can supplement the course, but no textbooks are required. All equipment needed will similarly be provided, except students will be expected to bring their own laptops. This class will have its last meeting day on Friday, Dec. 5, 2025.</t>
+  </si>
+  <si>
+    <t>The class will be a mixture of lecture, hands-on exercises, guest lectures from industry experts, and group learning and projects. NO PREREQUISITES ARE REQUIRED FOR THIS COURSE. All content and knowledge base required to be successful in this course will be covered and provided by the instructor. Optional textbooks can supplement the course, but no textbooks are required. All equipment needed will similarly be provided, except students will be expected to bring their own laptops.</t>
+  </si>
+  <si>
+    <t>Fall 2026, Spring 2026, Fall 2025</t>
   </si>
 </sst>
 </file>
@@ -8392,7 +8464,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -8406,6 +8478,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -8462,6 +8535,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8785,10 +8862,9 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.6328125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.81640625" style="1" customWidth="1"/>
-    <col min="3" max="4" width="10.81640625" style="1" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="10.81640625" style="3" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="11.54296875" style="1" hidden="1" customWidth="1"/>
+    <col min="2" max="4" width="10.81640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="10.81640625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="11.54296875" style="1" customWidth="1"/>
     <col min="7" max="7" width="62.6328125" style="1" customWidth="1"/>
     <col min="8" max="9" width="10.81640625" style="1" customWidth="1"/>
     <col min="10" max="15" width="22" style="1" customWidth="1"/>
@@ -19296,7 +19372,7 @@
         <v>1404</v>
       </c>
       <c r="G224" s="1" t="s">
-        <v>2514</v>
+        <v>2598</v>
       </c>
       <c r="H224" s="1" t="s">
         <v>1405</v>
@@ -19343,7 +19419,7 @@
         <v>1409</v>
       </c>
       <c r="G225" s="1" t="s">
-        <v>2514</v>
+        <v>2599</v>
       </c>
       <c r="H225" s="1" t="s">
         <v>1405</v>
@@ -19390,7 +19466,7 @@
         <v>268</v>
       </c>
       <c r="G226" s="1" t="s">
-        <v>2514</v>
+        <v>2596</v>
       </c>
       <c r="H226" s="1" t="s">
         <v>6</v>
@@ -19437,7 +19513,7 @@
         <v>1418</v>
       </c>
       <c r="G227" s="1" t="s">
-        <v>2514</v>
+        <v>46</v>
       </c>
       <c r="H227" s="1" t="s">
         <v>1419</v>
@@ -19484,7 +19560,7 @@
         <v>1424</v>
       </c>
       <c r="G228" s="1" t="s">
-        <v>2514</v>
+        <v>2598</v>
       </c>
       <c r="H228" s="1" t="s">
         <v>1425</v>
@@ -19531,7 +19607,7 @@
         <v>1430</v>
       </c>
       <c r="G229" s="1" t="s">
-        <v>2514</v>
+        <v>42</v>
       </c>
       <c r="H229" s="1" t="s">
         <v>1431</v>
@@ -19578,7 +19654,7 @@
         <v>1436</v>
       </c>
       <c r="G230" s="1" t="s">
-        <v>2514</v>
+        <v>2598</v>
       </c>
       <c r="H230" s="1" t="s">
         <v>1437</v>
@@ -19625,7 +19701,7 @@
         <v>344</v>
       </c>
       <c r="G231" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H231" s="1" t="s">
         <v>1442</v>
@@ -19672,7 +19748,7 @@
         <v>344</v>
       </c>
       <c r="G232" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H232" s="1" t="s">
         <v>1447</v>
@@ -19719,7 +19795,7 @@
         <v>344</v>
       </c>
       <c r="G233" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H233" s="1" t="s">
         <v>1452</v>
@@ -19766,7 +19842,7 @@
         <v>344</v>
       </c>
       <c r="G234" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H234" s="1" t="s">
         <v>1457</v>
@@ -19813,7 +19889,7 @@
         <v>1462</v>
       </c>
       <c r="G235" s="1" t="s">
-        <v>2514</v>
+        <v>42</v>
       </c>
       <c r="H235" s="1" t="s">
         <v>1463</v>
@@ -19860,7 +19936,7 @@
         <v>1022</v>
       </c>
       <c r="G236" s="1" t="s">
-        <v>2514</v>
+        <v>2597</v>
       </c>
       <c r="H236" s="1" t="s">
         <v>1468</v>
@@ -19907,7 +19983,7 @@
         <v>344</v>
       </c>
       <c r="G237" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H237" s="1" t="s">
         <v>1473</v>
@@ -19954,7 +20030,7 @@
         <v>1022</v>
       </c>
       <c r="G238" s="1" t="s">
-        <v>2514</v>
+        <v>2597</v>
       </c>
       <c r="H238" s="1" t="s">
         <v>1478</v>
@@ -20001,7 +20077,7 @@
         <v>1199</v>
       </c>
       <c r="G239" s="1" t="s">
-        <v>2514</v>
+        <v>43</v>
       </c>
       <c r="H239" s="1" t="s">
         <v>6</v>
@@ -20048,7 +20124,7 @@
         <v>344</v>
       </c>
       <c r="G240" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H240" s="1" t="s">
         <v>1488</v>
@@ -20095,7 +20171,7 @@
         <v>344</v>
       </c>
       <c r="G241" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H241" s="1" t="s">
         <v>1493</v>
@@ -20142,7 +20218,7 @@
         <v>344</v>
       </c>
       <c r="G242" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H242" s="1" t="s">
         <v>1498</v>
@@ -20189,7 +20265,7 @@
         <v>344</v>
       </c>
       <c r="G243" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H243" s="1" t="s">
         <v>1503</v>
@@ -20236,7 +20312,7 @@
         <v>344</v>
       </c>
       <c r="G244" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H244" s="1" t="s">
         <v>48</v>
@@ -20283,7 +20359,7 @@
         <v>1372</v>
       </c>
       <c r="G245" s="1" t="s">
-        <v>2514</v>
+        <v>2617</v>
       </c>
       <c r="H245" s="1" t="s">
         <v>6</v>
@@ -20330,7 +20406,7 @@
         <v>1372</v>
       </c>
       <c r="G246" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H246" s="1" t="s">
         <v>1515</v>
@@ -20377,7 +20453,7 @@
         <v>1372</v>
       </c>
       <c r="G247" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H247" s="1" t="s">
         <v>1515</v>
@@ -20424,7 +20500,7 @@
         <v>321</v>
       </c>
       <c r="G248" s="1" t="s">
-        <v>2514</v>
+        <v>2599</v>
       </c>
       <c r="H248" s="1" t="s">
         <v>321</v>
@@ -20459,7 +20535,7 @@
         <v>321</v>
       </c>
       <c r="G249" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H249" s="1" t="s">
         <v>321</v>
@@ -20494,7 +20570,7 @@
         <v>1531</v>
       </c>
       <c r="G250" s="1" t="s">
-        <v>2514</v>
+        <v>2618</v>
       </c>
       <c r="H250" s="1" t="s">
         <v>1532</v>
@@ -20541,7 +20617,7 @@
         <v>344</v>
       </c>
       <c r="G251" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H251" s="1" t="s">
         <v>1537</v>
@@ -20588,7 +20664,7 @@
         <v>218</v>
       </c>
       <c r="G252" s="1" t="s">
-        <v>2514</v>
+        <v>44</v>
       </c>
       <c r="H252" s="1" t="s">
         <v>1542</v>
@@ -20635,7 +20711,7 @@
         <v>344</v>
       </c>
       <c r="G253" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H253" s="1" t="s">
         <v>1547</v>
@@ -20682,7 +20758,7 @@
         <v>344</v>
       </c>
       <c r="G254" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H254" s="1" t="s">
         <v>1478</v>
@@ -20729,7 +20805,7 @@
         <v>344</v>
       </c>
       <c r="G255" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H255" s="1" t="s">
         <v>1542</v>
@@ -20776,7 +20852,7 @@
         <v>344</v>
       </c>
       <c r="G256" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H256" s="1" t="s">
         <v>1488</v>
@@ -20823,7 +20899,7 @@
         <v>1564</v>
       </c>
       <c r="G257" s="1" t="s">
-        <v>2514</v>
+        <v>2619</v>
       </c>
       <c r="H257" s="1" t="s">
         <v>6</v>
@@ -20870,7 +20946,7 @@
         <v>1569</v>
       </c>
       <c r="G258" s="1" t="s">
-        <v>2514</v>
+        <v>2599</v>
       </c>
       <c r="H258" s="1" t="s">
         <v>1570</v>
@@ -20917,7 +20993,7 @@
         <v>1569</v>
       </c>
       <c r="G259" s="1" t="s">
-        <v>2514</v>
+        <v>2599</v>
       </c>
       <c r="H259" s="1" t="s">
         <v>1575</v>
@@ -20964,7 +21040,7 @@
         <v>344</v>
       </c>
       <c r="G260" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H260" s="1" t="s">
         <v>48</v>
@@ -21011,7 +21087,7 @@
         <v>344</v>
       </c>
       <c r="G261" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H261" s="1" t="s">
         <v>1584</v>
@@ -21058,7 +21134,7 @@
         <v>1378</v>
       </c>
       <c r="G262" s="1" t="s">
-        <v>2514</v>
+        <v>45</v>
       </c>
       <c r="H262" s="1" t="s">
         <v>1589</v>
@@ -21105,7 +21181,7 @@
         <v>344</v>
       </c>
       <c r="G263" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H263" s="1" t="s">
         <v>1594</v>
@@ -21152,7 +21228,7 @@
         <v>1599</v>
       </c>
       <c r="G264" s="1" t="s">
-        <v>2514</v>
+        <v>2599</v>
       </c>
       <c r="H264" s="1" t="s">
         <v>1600</v>
@@ -21199,7 +21275,7 @@
         <v>344</v>
       </c>
       <c r="G265" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H265" s="1" t="s">
         <v>6</v>
@@ -21246,7 +21322,7 @@
         <v>1372</v>
       </c>
       <c r="G266" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H266" s="1" t="s">
         <v>6</v>
@@ -21293,7 +21369,7 @@
         <v>1611</v>
       </c>
       <c r="G267" s="1" t="s">
-        <v>2514</v>
+        <v>2617</v>
       </c>
       <c r="H267" s="1" t="s">
         <v>6</v>
@@ -21340,7 +21416,7 @@
         <v>344</v>
       </c>
       <c r="G268" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H268" s="1" t="s">
         <v>1616</v>
@@ -21387,7 +21463,7 @@
         <v>1622</v>
       </c>
       <c r="G269" s="1" t="s">
-        <v>2514</v>
+        <v>2617</v>
       </c>
       <c r="H269" s="1" t="s">
         <v>1616</v>
@@ -21434,7 +21510,7 @@
         <v>1628</v>
       </c>
       <c r="G270" s="1" t="s">
-        <v>2514</v>
+        <v>2617</v>
       </c>
       <c r="H270" s="1" t="s">
         <v>1629</v>
@@ -21481,7 +21557,7 @@
         <v>1628</v>
       </c>
       <c r="G271" s="1" t="s">
-        <v>2514</v>
+        <v>2617</v>
       </c>
       <c r="H271" s="1" t="s">
         <v>1635</v>
@@ -21528,7 +21604,7 @@
         <v>1628</v>
       </c>
       <c r="G272" s="1" t="s">
-        <v>2514</v>
+        <v>2617</v>
       </c>
       <c r="H272" s="1" t="s">
         <v>1641</v>
@@ -21575,7 +21651,7 @@
         <v>1628</v>
       </c>
       <c r="G273" s="1" t="s">
-        <v>2514</v>
+        <v>2617</v>
       </c>
       <c r="H273" s="1" t="s">
         <v>1647</v>
@@ -21622,7 +21698,7 @@
         <v>1652</v>
       </c>
       <c r="G274" s="1" t="s">
-        <v>2514</v>
+        <v>2618</v>
       </c>
       <c r="H274" s="1" t="s">
         <v>1653</v>
@@ -21669,7 +21745,7 @@
         <v>1652</v>
       </c>
       <c r="G275" s="1" t="s">
-        <v>2514</v>
+        <v>2617</v>
       </c>
       <c r="H275" s="1" t="s">
         <v>1658</v>
@@ -21716,7 +21792,7 @@
         <v>1652</v>
       </c>
       <c r="G276" s="1" t="s">
-        <v>2514</v>
+        <v>2617</v>
       </c>
       <c r="H276" s="1" t="s">
         <v>1663</v>
@@ -21763,7 +21839,7 @@
         <v>1669</v>
       </c>
       <c r="G277" s="1" t="s">
-        <v>2514</v>
+        <v>2617</v>
       </c>
       <c r="H277" s="1" t="s">
         <v>1670</v>
@@ -21810,7 +21886,7 @@
         <v>1652</v>
       </c>
       <c r="G278" s="1" t="s">
-        <v>2514</v>
+        <v>2617</v>
       </c>
       <c r="H278" s="1" t="s">
         <v>1675</v>
@@ -21857,7 +21933,7 @@
         <v>1680</v>
       </c>
       <c r="G279" s="1" t="s">
-        <v>2514</v>
+        <v>2620</v>
       </c>
       <c r="H279" s="1" t="s">
         <v>1681</v>
@@ -21904,7 +21980,7 @@
         <v>1652</v>
       </c>
       <c r="G280" s="1" t="s">
-        <v>2514</v>
+        <v>2621</v>
       </c>
       <c r="H280" s="1" t="s">
         <v>1686</v>
@@ -21951,7 +22027,7 @@
         <v>344</v>
       </c>
       <c r="G281" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H281" s="1" t="s">
         <v>1690</v>
@@ -21998,7 +22074,7 @@
         <v>1652</v>
       </c>
       <c r="G282" s="1" t="s">
-        <v>2514</v>
+        <v>2617</v>
       </c>
       <c r="H282" s="1" t="s">
         <v>1695</v>
@@ -22045,7 +22121,7 @@
         <v>1652</v>
       </c>
       <c r="G283" s="1" t="s">
-        <v>2514</v>
+        <v>2618</v>
       </c>
       <c r="H283" s="1" t="s">
         <v>1700</v>
@@ -22092,7 +22168,7 @@
         <v>1652</v>
       </c>
       <c r="G284" s="1" t="s">
-        <v>2514</v>
+        <v>2617</v>
       </c>
       <c r="H284" s="1" t="s">
         <v>1705</v>
@@ -22139,7 +22215,7 @@
         <v>1652</v>
       </c>
       <c r="G285" s="1" t="s">
-        <v>2514</v>
+        <v>2598</v>
       </c>
       <c r="H285" s="1" t="s">
         <v>1710</v>
@@ -22186,7 +22262,7 @@
         <v>1652</v>
       </c>
       <c r="G286" s="1" t="s">
-        <v>2514</v>
+        <v>2622</v>
       </c>
       <c r="H286" s="1" t="s">
         <v>1714</v>
@@ -22233,7 +22309,7 @@
         <v>1652</v>
       </c>
       <c r="G287" s="1" t="s">
-        <v>2514</v>
+        <v>2617</v>
       </c>
       <c r="H287" s="1" t="s">
         <v>1719</v>
@@ -22280,7 +22356,7 @@
         <v>1680</v>
       </c>
       <c r="G288" s="1" t="s">
-        <v>2514</v>
+        <v>2623</v>
       </c>
       <c r="H288" s="1" t="s">
         <v>1670</v>
@@ -22327,7 +22403,7 @@
         <v>1652</v>
       </c>
       <c r="G289" s="1" t="s">
-        <v>2514</v>
+        <v>2624</v>
       </c>
       <c r="H289" s="1" t="s">
         <v>1726</v>
@@ -22374,7 +22450,7 @@
         <v>514</v>
       </c>
       <c r="G290" s="1" t="s">
-        <v>2514</v>
+        <v>2625</v>
       </c>
       <c r="H290" s="1" t="s">
         <v>1616</v>
@@ -22421,7 +22497,7 @@
         <v>1735</v>
       </c>
       <c r="G291" s="1" t="s">
-        <v>2514</v>
+        <v>43</v>
       </c>
       <c r="H291" s="1" t="s">
         <v>1736</v>
@@ -22468,7 +22544,7 @@
         <v>344</v>
       </c>
       <c r="G292" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H292" s="1" t="s">
         <v>48</v>
@@ -22515,7 +22591,7 @@
         <v>1744</v>
       </c>
       <c r="G293" s="1" t="s">
-        <v>2514</v>
+        <v>42</v>
       </c>
       <c r="H293" s="1" t="s">
         <v>1745</v>
@@ -22562,7 +22638,7 @@
         <v>1744</v>
       </c>
       <c r="G294" s="1" t="s">
-        <v>2514</v>
+        <v>42</v>
       </c>
       <c r="H294" s="1" t="s">
         <v>1745</v>
@@ -22609,7 +22685,7 @@
         <v>344</v>
       </c>
       <c r="G295" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H295" s="1" t="s">
         <v>1752</v>
@@ -22656,7 +22732,7 @@
         <v>344</v>
       </c>
       <c r="G296" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H296" s="1" t="s">
         <v>1752</v>
@@ -22703,7 +22779,7 @@
         <v>1760</v>
       </c>
       <c r="G297" s="1" t="s">
-        <v>2514</v>
+        <v>2626</v>
       </c>
       <c r="H297" s="1" t="s">
         <v>1761</v>
@@ -22750,7 +22826,7 @@
         <v>1765</v>
       </c>
       <c r="G298" s="1" t="s">
-        <v>2514</v>
+        <v>2597</v>
       </c>
       <c r="H298" s="1" t="s">
         <v>1766</v>
@@ -22797,7 +22873,7 @@
         <v>344</v>
       </c>
       <c r="G299" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H299" s="1" t="s">
         <v>1770</v>
@@ -22844,7 +22920,7 @@
         <v>344</v>
       </c>
       <c r="G300" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H300" s="1" t="s">
         <v>6</v>
@@ -22891,7 +22967,7 @@
         <v>344</v>
       </c>
       <c r="G301" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H301" s="1" t="s">
         <v>402</v>
@@ -22938,7 +23014,7 @@
         <v>344</v>
       </c>
       <c r="G302" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H302" s="1" t="s">
         <v>402</v>
@@ -22985,7 +23061,7 @@
         <v>1786</v>
       </c>
       <c r="G303" s="1" t="s">
-        <v>2514</v>
+        <v>42</v>
       </c>
       <c r="H303" s="1" t="s">
         <v>1787</v>
@@ -23032,7 +23108,7 @@
         <v>344</v>
       </c>
       <c r="G304" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H304" s="1" t="s">
         <v>1791</v>
@@ -23079,7 +23155,7 @@
         <v>344</v>
       </c>
       <c r="G305" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H305" s="1" t="s">
         <v>1796</v>
@@ -23126,7 +23202,7 @@
         <v>344</v>
       </c>
       <c r="G306" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H306" s="1" t="s">
         <v>1801</v>
@@ -23173,7 +23249,7 @@
         <v>344</v>
       </c>
       <c r="G307" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H307" s="1" t="s">
         <v>1806</v>
@@ -23220,7 +23296,7 @@
         <v>344</v>
       </c>
       <c r="G308" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H308" s="1" t="s">
         <v>1801</v>
@@ -23267,7 +23343,7 @@
         <v>344</v>
       </c>
       <c r="G309" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H309" s="1" t="s">
         <v>48</v>
@@ -23314,7 +23390,7 @@
         <v>344</v>
       </c>
       <c r="G310" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H310" s="1" t="s">
         <v>1820</v>
@@ -23361,7 +23437,7 @@
         <v>1825</v>
       </c>
       <c r="G311" s="1" t="s">
-        <v>2514</v>
+        <v>2627</v>
       </c>
       <c r="H311" s="1" t="s">
         <v>6</v>
@@ -23408,7 +23484,7 @@
         <v>344</v>
       </c>
       <c r="G312" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H312" s="1" t="s">
         <v>1830</v>
@@ -23455,7 +23531,7 @@
         <v>344</v>
       </c>
       <c r="G313" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H313" s="1" t="s">
         <v>1835</v>
@@ -23502,7 +23578,7 @@
         <v>1840</v>
       </c>
       <c r="G314" s="1" t="s">
-        <v>2514</v>
+        <v>42</v>
       </c>
       <c r="H314" s="1" t="s">
         <v>48</v>
@@ -23549,7 +23625,7 @@
         <v>344</v>
       </c>
       <c r="G315" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H315" s="1" t="s">
         <v>1844</v>
@@ -23596,7 +23672,7 @@
         <v>344</v>
       </c>
       <c r="G316" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H316" s="1" t="s">
         <v>1009</v>
@@ -23643,7 +23719,7 @@
         <v>514</v>
       </c>
       <c r="G317" s="1" t="s">
-        <v>2514</v>
+        <v>2630</v>
       </c>
       <c r="H317" s="1" t="s">
         <v>6</v>
@@ -23690,7 +23766,7 @@
         <v>344</v>
       </c>
       <c r="G318" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H318" s="1" t="s">
         <v>402</v>
@@ -23737,7 +23813,7 @@
         <v>344</v>
       </c>
       <c r="G319" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H319" s="1" t="s">
         <v>402</v>
@@ -23784,7 +23860,7 @@
         <v>344</v>
       </c>
       <c r="G320" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H320" s="1" t="s">
         <v>402</v>
@@ -23831,7 +23907,7 @@
         <v>344</v>
       </c>
       <c r="G321" s="1" t="s">
-        <v>2514</v>
+        <v>2616</v>
       </c>
       <c r="H321" s="1" t="s">
         <v>1864</v>
@@ -28954,7 +29030,7 @@
         <v>377</v>
       </c>
       <c r="G430" s="1" t="s">
-        <v>2514</v>
+        <v>2600</v>
       </c>
       <c r="H430" s="1" t="s">
         <v>2291</v>
@@ -29001,7 +29077,7 @@
         <v>2296</v>
       </c>
       <c r="G431" s="1" t="s">
-        <v>2514</v>
+        <v>2596</v>
       </c>
       <c r="H431" s="1" t="s">
         <v>2297</v>
@@ -29048,7 +29124,7 @@
         <v>425</v>
       </c>
       <c r="G432" s="1" t="s">
-        <v>2514</v>
+        <v>2600</v>
       </c>
       <c r="H432" s="1" t="s">
         <v>6</v>
@@ -29095,7 +29171,7 @@
         <v>1077</v>
       </c>
       <c r="G433" s="1" t="s">
-        <v>2514</v>
+        <v>2628</v>
       </c>
       <c r="H433" s="1" t="s">
         <v>2305</v>
@@ -29142,7 +29218,7 @@
         <v>268</v>
       </c>
       <c r="G434" s="1" t="s">
-        <v>2514</v>
+        <v>46</v>
       </c>
       <c r="H434" s="1" t="s">
         <v>2309</v>
@@ -29377,7 +29453,7 @@
         <v>514</v>
       </c>
       <c r="G439" s="1" t="s">
-        <v>2514</v>
+        <v>2639</v>
       </c>
       <c r="H439" s="1" t="s">
         <v>296</v>
@@ -29464,7 +29540,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B785887B-576B-4D81-AE70-D107EA8277F5}">
-  <dimension ref="A1:R134"/>
+  <dimension ref="A1:R137"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="9.81640625" customWidth="1"/>
@@ -36579,6 +36655,165 @@
       </c>
       <c r="Q134" t="s">
         <v>181</v>
+      </c>
+    </row>
+    <row r="135" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A135" t="s">
+        <v>2629</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>1849</v>
+      </c>
+      <c r="C135" t="s">
+        <v>44</v>
+      </c>
+      <c r="D135" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E135" t="s">
+        <v>2633</v>
+      </c>
+      <c r="F135" t="s">
+        <v>2636</v>
+      </c>
+      <c r="G135" s="4">
+        <v>3</v>
+      </c>
+      <c r="H135" s="7" t="s">
+        <v>2637</v>
+      </c>
+      <c r="I135" t="s">
+        <v>2630</v>
+      </c>
+      <c r="J135" t="s">
+        <v>6</v>
+      </c>
+      <c r="K135" t="s">
+        <v>2514</v>
+      </c>
+      <c r="L135" s="4" t="s">
+        <v>2462</v>
+      </c>
+      <c r="M135" t="s">
+        <v>2434</v>
+      </c>
+      <c r="N135" t="s">
+        <v>2452</v>
+      </c>
+      <c r="O135" t="s">
+        <v>2434</v>
+      </c>
+      <c r="P135" t="s">
+        <v>2434</v>
+      </c>
+      <c r="Q135" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="136" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A136" t="s">
+        <v>2631</v>
+      </c>
+      <c r="B136" s="1" t="s">
+        <v>1849</v>
+      </c>
+      <c r="C136" t="s">
+        <v>43</v>
+      </c>
+      <c r="D136" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E136" t="s">
+        <v>2633</v>
+      </c>
+      <c r="F136" t="s">
+        <v>2634</v>
+      </c>
+      <c r="G136" s="4">
+        <v>3</v>
+      </c>
+      <c r="H136" s="7" t="s">
+        <v>2635</v>
+      </c>
+      <c r="I136" t="s">
+        <v>2630</v>
+      </c>
+      <c r="J136" t="s">
+        <v>6</v>
+      </c>
+      <c r="K136" t="s">
+        <v>2514</v>
+      </c>
+      <c r="L136" s="4" t="s">
+        <v>2462</v>
+      </c>
+      <c r="M136" t="s">
+        <v>2434</v>
+      </c>
+      <c r="N136" t="s">
+        <v>2452</v>
+      </c>
+      <c r="O136" t="s">
+        <v>2434</v>
+      </c>
+      <c r="P136" t="s">
+        <v>2434</v>
+      </c>
+      <c r="Q136" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="137" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A137" t="s">
+        <v>2632</v>
+      </c>
+      <c r="B137" s="1" t="s">
+        <v>1849</v>
+      </c>
+      <c r="C137" t="s">
+        <v>42</v>
+      </c>
+      <c r="D137" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E137" t="s">
+        <v>2633</v>
+      </c>
+      <c r="F137" t="s">
+        <v>2636</v>
+      </c>
+      <c r="G137" s="4">
+        <v>3</v>
+      </c>
+      <c r="H137" s="7" t="s">
+        <v>2638</v>
+      </c>
+      <c r="I137" t="s">
+        <v>2630</v>
+      </c>
+      <c r="J137" t="s">
+        <v>6</v>
+      </c>
+      <c r="K137" t="s">
+        <v>2514</v>
+      </c>
+      <c r="L137" s="4" t="s">
+        <v>2462</v>
+      </c>
+      <c r="M137" t="s">
+        <v>2434</v>
+      </c>
+      <c r="N137" t="s">
+        <v>2452</v>
+      </c>
+      <c r="O137" t="s">
+        <v>2434</v>
+      </c>
+      <c r="P137" t="s">
+        <v>2434</v>
+      </c>
+      <c r="Q137" t="s">
+        <v>2557</v>
       </c>
     </row>
   </sheetData>

</xml_diff>